<commit_message>
Nubank: conserta o acento embaralhado da exportação
A fatura de março, com 156 lançamentos, foi lida em sandbox: 145 compras,
o pagamento da fatura anterior indo para Transferências entre Contas (e não
para receita), 41 parcelas reconhecidas e uma duplicidade provável — a mesma
academia cobrada duas vezes no mesmo dia pelo mesmo valor, que fica para o
André decidir.

O único defeito era de texto: a exportação do Nubank grava em UTF-8 e declara
latin-1, então nenhum acento chega inteiro ("Ajuste a crÃ©dito"). O conserto
vale na entrada, não só na tela: a memória de estabelecimentos guarda a
descrição, e as duas grafias virariam chaves diferentes para o mesmo lugar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7Qj4WdRQsN9svxJDqzufY
</commit_message>
<xml_diff>
--- a/tests/amostras/nubank_fatura.xlsx
+++ b/tests/amostras/nubank_fatura.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,6 +637,23 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-03-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ajuste a crÃ©dito</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>-19.3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>